<commit_message>
Refactoring and updated README
</commit_message>
<xml_diff>
--- a/data/Inventory.xlsx
+++ b/data/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9060"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Lembar1" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>Stok</t>
   </si>
   <si>
-    <t>NG001</t>
+    <t>001</t>
   </si>
   <si>
     <t>Indomie Goreng</t>
@@ -53,31 +53,31 @@
     <t>Makanan</t>
   </si>
   <si>
-    <t>NG002</t>
+    <t>002</t>
   </si>
   <si>
     <t>Indomie Soto</t>
   </si>
   <si>
-    <t>NG003</t>
+    <t>003</t>
   </si>
   <si>
     <t>Roti Tawar</t>
   </si>
   <si>
-    <t>NG004</t>
+    <t>004</t>
   </si>
   <si>
     <t>Biskuit Roma Kelapa</t>
   </si>
   <si>
-    <t>NG005</t>
+    <t>005</t>
   </si>
   <si>
     <t>Chitato Sapi Panggang</t>
   </si>
   <si>
-    <t>NG006</t>
+    <t>006</t>
   </si>
   <si>
     <t>Aqua 600ml</t>
@@ -86,31 +86,31 @@
     <t>Minuman</t>
   </si>
   <si>
-    <t>NG007</t>
+    <t>007</t>
   </si>
   <si>
     <t>Teh Botol Sostro</t>
   </si>
   <si>
-    <t>NG008</t>
+    <t>008</t>
   </si>
   <si>
     <t>Pocari Sweat 500ml</t>
   </si>
   <si>
-    <t>NG009</t>
+    <t>009</t>
   </si>
   <si>
     <t>Kopi Good Day</t>
   </si>
   <si>
-    <t>NG010</t>
+    <t>010</t>
   </si>
   <si>
     <t>Susu Ultra Milk 1L</t>
   </si>
   <si>
-    <t>NG011</t>
+    <t>011</t>
   </si>
   <si>
     <t>Beras Premium 5kg</t>
@@ -119,31 +119,31 @@
     <t>Sembako</t>
   </si>
   <si>
-    <t>NG012</t>
+    <t>012</t>
   </si>
   <si>
     <t>Minyak Goreng 1L</t>
   </si>
   <si>
-    <t>NG013</t>
+    <t>013</t>
   </si>
   <si>
     <t>Gula Pasir 1kg</t>
   </si>
   <si>
-    <t>NG014</t>
+    <t>014</t>
   </si>
   <si>
     <t>Tepung Terigu 1kg</t>
   </si>
   <si>
-    <t>NG015</t>
+    <t>015</t>
   </si>
   <si>
     <t>Telur Ayam 1kg</t>
   </si>
   <si>
-    <t>NG016</t>
+    <t>016</t>
   </si>
   <si>
     <t>Sabun Lifebuoy</t>
@@ -152,7 +152,7 @@
     <t>Kebersihan</t>
   </si>
   <si>
-    <t>NG017</t>
+    <t>017</t>
   </si>
   <si>
     <t>Shampoo Sunsilk</t>
@@ -161,25 +161,25 @@
     <t>Perawatan</t>
   </si>
   <si>
-    <t>NG018</t>
+    <t>018</t>
   </si>
   <si>
     <t>Pasta Gigi Pepsodent</t>
   </si>
   <si>
-    <t>NG019</t>
+    <t>019</t>
   </si>
   <si>
     <t>Sabun Cuci Piring Sunlight</t>
   </si>
   <si>
-    <t>NG020</t>
+    <t>020</t>
   </si>
   <si>
     <t>Deterjen Rinso 800g</t>
   </si>
   <si>
-    <t>NG021</t>
+    <t>021</t>
   </si>
   <si>
     <t>Pulpen Standard AE7</t>
@@ -188,31 +188,31 @@
     <t>ATK</t>
   </si>
   <si>
-    <t>NG022</t>
+    <t>022</t>
   </si>
   <si>
     <t>Buku Tulis 58 Lembar</t>
   </si>
   <si>
-    <t>NG023</t>
+    <t>023</t>
   </si>
   <si>
     <t>Pensil 2B</t>
   </si>
   <si>
-    <t>NG024</t>
+    <t>024</t>
   </si>
   <si>
     <t>Penghapus</t>
   </si>
   <si>
-    <t>NG025</t>
+    <t>025</t>
   </si>
   <si>
     <t>Spidol Snowman</t>
   </si>
   <si>
-    <t>NG026</t>
+    <t>026</t>
   </si>
   <si>
     <t>Kabel Data USB Type-C</t>
@@ -221,25 +221,25 @@
     <t>Elektronik</t>
   </si>
   <si>
-    <t>NG027</t>
+    <t>027</t>
   </si>
   <si>
     <t>Baterai AA 2pcs</t>
   </si>
   <si>
-    <t>NG028</t>
+    <t>028</t>
   </si>
   <si>
     <t>Lampu Led 9 Watt</t>
   </si>
   <si>
-    <t>NG029</t>
+    <t>029</t>
   </si>
   <si>
     <t>Tisu Wajah 200 Lembar</t>
   </si>
   <si>
-    <t>NG030</t>
+    <t>030</t>
   </si>
   <si>
     <t>Pewangi Ruangan</t>
@@ -858,8 +858,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1390,7 +1393,7 @@
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="7.22222222222222" customWidth="1"/>
+    <col min="1" max="1" width="7.22222222222222" style="1" customWidth="1"/>
     <col min="2" max="2" width="23.1111111111111" customWidth="1"/>
     <col min="3" max="3" width="10.6666666666667" customWidth="1"/>
     <col min="4" max="4" width="6.66666666666667" customWidth="1"/>
@@ -1398,7 +1401,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1415,7 +1418,7 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
@@ -1432,7 +1435,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
@@ -1449,7 +1452,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B4" t="s">
@@ -1466,7 +1469,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B5" t="s">
@@ -1483,7 +1486,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
@@ -1500,7 +1503,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7" t="s">
@@ -1517,7 +1520,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B8" t="s">
@@ -1534,7 +1537,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B9" t="s">
@@ -1551,7 +1554,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B10" t="s">
@@ -1568,7 +1571,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B11" t="s">
@@ -1585,7 +1588,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B12" t="s">
@@ -1602,7 +1605,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B13" t="s">
@@ -1619,7 +1622,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B14" t="s">
@@ -1636,7 +1639,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B15" t="s">
@@ -1653,7 +1656,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B16" t="s">
@@ -1670,7 +1673,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B17" t="s">
@@ -1687,7 +1690,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B18" t="s">
@@ -1704,7 +1707,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B19" t="s">
@@ -1721,7 +1724,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B20" t="s">
@@ -1738,7 +1741,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B21" t="s">
@@ -1755,7 +1758,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" t="s">
+      <c r="A22" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B22" t="s">
@@ -1772,7 +1775,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" t="s">
+      <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B23" t="s">
@@ -1789,7 +1792,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" t="s">
+      <c r="A24" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B24" t="s">
@@ -1806,7 +1809,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" t="s">
+      <c r="A25" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B25" t="s">
@@ -1823,7 +1826,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" t="s">
+      <c r="A26" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B26" t="s">
@@ -1840,7 +1843,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" t="s">
+      <c r="A27" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B27" t="s">
@@ -1857,7 +1860,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" t="s">
+      <c r="A28" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B28" t="s">
@@ -1874,7 +1877,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" t="s">
+      <c r="A29" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B29" t="s">
@@ -1891,7 +1894,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" t="s">
+      <c r="A30" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B30" t="s">
@@ -1908,7 +1911,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" t="s">
+      <c r="A31" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B31" t="s">

</xml_diff>

<commit_message>
Rename Neon Market to Neon Store
</commit_message>
<xml_diff>
--- a/data/Inventory.xlsx
+++ b/data/Inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="E16" t="n">
         <v>15</v>
@@ -1113,6 +1113,27 @@
       </c>
       <c r="E33" t="n">
         <v>75</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>34</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Aqua Galon</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Minuman</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E34" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>